<commit_message>
1.0.5 — Monthly expenses live in the settings, the Expenses sheet is no longer read
Only the sheet "Data Input" is read. The eight targets are multiples of
one setting, monthlyExpenses (default 2 500 a month, an estimate until
touched). Importer, store, calc, settings pane, example workbook, tests
and docs follow; MODEL_VERSION 3 discards stored models of the old shape.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/nordstern-example.xlsx
+++ b/examples/nordstern-example.xlsx
@@ -15,7 +15,6 @@
   <sheets>
     <sheet name="Read me" sheetId="1" r:id="rId1"/>
     <sheet name="Data Input" sheetId="2" r:id="rId2"/>
-    <sheet name="Expenses" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -35,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="46">
   <si>
     <t>NORDSTERN — example workbook</t>
   </si>
@@ -49,7 +48,7 @@
     <t>all of it, so the numbers show a large asset and a large debt side by side.</t>
   </si>
   <si>
-    <t>nordstern reads two sheets and nothing else:</t>
+    <t>nordstern reads one sheet and nothing else:</t>
   </si>
   <si>
     <t xml:space="preserve">  "Data Input"</t>
@@ -58,13 +57,7 @@
     <t>one column per month, one row per account</t>
   </si>
   <si>
-    <t xml:space="preserve">  "Expenses"</t>
-  </si>
-  <si>
-    <t>your fixed costs, monthly and annual</t>
-  </si>
-  <si>
-    <t>This third sheet is here to prove the point: it is never read.</t>
+    <t>This second sheet is here to prove the point: it is never read.</t>
   </si>
   <si>
     <t>Add as many of your own as you like.</t>
@@ -179,105 +172,6 @@
   </si>
   <si>
     <t>Total net worth</t>
-  </si>
-  <si>
-    <t>Kind</t>
-  </si>
-  <si>
-    <t>Amount</t>
-  </si>
-  <si>
-    <t>Due</t>
-  </si>
-  <si>
-    <t>Mortgage (interest + amortisation)</t>
-  </si>
-  <si>
-    <t>monthly</t>
-  </si>
-  <si>
-    <t>Service charges (owners’ association)</t>
-  </si>
-  <si>
-    <t>Securities loan interest</t>
-  </si>
-  <si>
-    <t>Electricity</t>
-  </si>
-  <si>
-    <t>Internet</t>
-  </si>
-  <si>
-    <t>Mobile phone</t>
-  </si>
-  <si>
-    <t>Groceries</t>
-  </si>
-  <si>
-    <t>Public transport</t>
-  </si>
-  <si>
-    <t>Gym</t>
-  </si>
-  <si>
-    <t>Streaming</t>
-  </si>
-  <si>
-    <t>Dental top-up</t>
-  </si>
-  <si>
-    <t>Monthly fixed costs</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>Property tax</t>
-  </si>
-  <si>
-    <t>February</t>
-  </si>
-  <si>
-    <t>Car insurance</t>
-  </si>
-  <si>
-    <t>January</t>
-  </si>
-  <si>
-    <t>Car tax</t>
-  </si>
-  <si>
-    <t>March</t>
-  </si>
-  <si>
-    <t>Home contents insurance</t>
-  </si>
-  <si>
-    <t>April</t>
-  </si>
-  <si>
-    <t>Liability insurance</t>
-  </si>
-  <si>
-    <t>Broadcasting fee</t>
-  </si>
-  <si>
-    <t>quarterly</t>
-  </si>
-  <si>
-    <t>Travel health insurance</t>
-  </si>
-  <si>
-    <t>June</t>
-  </si>
-  <si>
-    <t>Software licences</t>
-  </si>
-  <si>
-    <t>November</t>
-  </si>
-  <si>
-    <t>Annual fixed costs</t>
   </si>
 </sst>
 </file>
@@ -795,37 +689,29 @@
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A9" t="s">
-        <v>7</v>
-      </c>
-      <c r="B9" t="s">
-        <v>8</v>
-      </c>
-    </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
   </sheetData>
@@ -847,7 +733,7 @@
   <sheetData>
     <row r="1" spans="1:85" s="4" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1" s="4" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B1" s="18">
         <v>43738</v>
@@ -1104,12 +990,12 @@
     </row>
     <row r="3" spans="1:85" s="16" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A3" s="15" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="4" spans="1:85" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B4" s="1">
         <v>4682.37</v>
@@ -1366,7 +1252,7 @@
     </row>
     <row r="5" spans="1:85" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B5" s="1">
         <v>4703.2</v>
@@ -1623,7 +1509,7 @@
     </row>
     <row r="6" spans="1:85" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B6" s="1">
         <v>1749.51</v>
@@ -1880,7 +1766,7 @@
     </row>
     <row r="7" spans="1:85" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B7" s="1">
         <v>812.83</v>
@@ -2137,7 +2023,7 @@
     </row>
     <row r="8" spans="1:85" s="15" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A8" s="15" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B8" s="17">
         <f>SUM(B4:B7)</f>
@@ -2478,12 +2364,12 @@
     </row>
     <row r="10" spans="1:85" s="8" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
     <row r="11" spans="1:85" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B11" s="1">
         <v>118</v>
@@ -2740,7 +2626,7 @@
     </row>
     <row r="12" spans="1:85" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B12" s="1">
         <v>0</v>
@@ -2997,7 +2883,7 @@
     </row>
     <row r="13" spans="1:85" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B13" s="1">
         <v>0</v>
@@ -3254,7 +3140,7 @@
     </row>
     <row r="14" spans="1:85" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B14" s="3">
         <f>SUM(B11:B13)</f>
@@ -3595,12 +3481,12 @@
     </row>
     <row r="16" spans="1:85" s="14" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A16" s="12" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="17" spans="1:85" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B17" s="1">
         <v>8342.52</v>
@@ -3857,7 +3743,7 @@
     </row>
     <row r="18" spans="1:85" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B18" s="1">
         <v>4538.6000000000004</v>
@@ -4114,7 +4000,7 @@
     </row>
     <row r="19" spans="1:85" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B19" s="1">
         <v>2664.91</v>
@@ -4371,7 +4257,7 @@
     </row>
     <row r="20" spans="1:85" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B20" s="1">
         <v>1544.11</v>
@@ -4628,7 +4514,7 @@
     </row>
     <row r="21" spans="1:85" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B21" s="1">
         <v>2249.12</v>
@@ -4885,7 +4771,7 @@
     </row>
     <row r="22" spans="1:85" s="12" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A22" s="12" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B22" s="13">
         <f>SUM(B17:B21)</f>
@@ -5226,12 +5112,12 @@
     </row>
     <row r="24" spans="1:85" s="11" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A24" s="9" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="25" spans="1:85" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B25" s="1">
         <v>410000</v>
@@ -5488,7 +5374,7 @@
     </row>
     <row r="26" spans="1:85" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B26" s="1">
         <v>26000</v>
@@ -5745,7 +5631,7 @@
     </row>
     <row r="27" spans="1:85" s="9" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A27" s="9" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B27" s="10">
         <f>SUM(B25:B26)</f>
@@ -6086,12 +5972,12 @@
     </row>
     <row r="29" spans="1:85" s="8" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A29" s="2" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
     </row>
     <row r="30" spans="1:85" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B30" s="1">
         <v>11793.26</v>
@@ -6348,7 +6234,7 @@
     </row>
     <row r="31" spans="1:85" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B31" s="1">
         <v>6312.88</v>
@@ -6605,7 +6491,7 @@
     </row>
     <row r="32" spans="1:85" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A32" s="2" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B32" s="3">
         <f>SUM(B30:B31)</f>
@@ -6947,7 +6833,7 @@
     <row r="33" spans="1:85" s="23" customFormat="1" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="34" spans="1:85" s="19" customFormat="1" ht="17" thickTop="1" x14ac:dyDescent="0.2">
       <c r="A34" s="19" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B34" s="20">
         <f>SUM(B8,B14,B22,B27,B32)</f>
@@ -7288,12 +7174,12 @@
     </row>
     <row r="36" spans="1:85" s="7" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A36" s="5" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="37" spans="1:85" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B37" s="1">
         <v>409145.84</v>
@@ -7550,7 +7436,7 @@
     </row>
     <row r="38" spans="1:85" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B38" s="1">
         <v>0</v>
@@ -7807,7 +7693,7 @@
     </row>
     <row r="39" spans="1:85" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B39" s="1">
         <v>710.52</v>
@@ -8064,7 +7950,7 @@
     </row>
     <row r="40" spans="1:85" s="5" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A40" s="5" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B40" s="6">
         <f>SUM(B37:B39)</f>
@@ -8406,7 +8292,7 @@
     <row r="41" spans="1:85" s="23" customFormat="1" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="42" spans="1:85" s="21" customFormat="1" ht="17" thickTop="1" x14ac:dyDescent="0.2">
       <c r="A42" s="21" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B42" s="22">
         <f>B34-B40</f>
@@ -8751,263 +8637,4 @@
     <ignoredError sqref="A1:CG7 A9:CG13 A8 A15:CG21 A14 A23:CG26 A22 A28:CG31 A27 A33:CG33 A32 A35:CG39 A34 A41:CG41 A40 A42" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:C23"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="1" width="34.83203125" customWidth="1"/>
-    <col min="2" max="3" width="12.83203125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
-        <v>48</v>
-      </c>
-      <c r="B1" t="s">
-        <v>49</v>
-      </c>
-      <c r="C1" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>51</v>
-      </c>
-      <c r="B2" s="1">
-        <v>1708.33</v>
-      </c>
-      <c r="C2" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>53</v>
-      </c>
-      <c r="B3" s="1">
-        <v>385</v>
-      </c>
-      <c r="C3" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>54</v>
-      </c>
-      <c r="B4" s="1">
-        <v>291.67</v>
-      </c>
-      <c r="C4" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
-        <v>55</v>
-      </c>
-      <c r="B5" s="1">
-        <v>78</v>
-      </c>
-      <c r="C5" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
-        <v>56</v>
-      </c>
-      <c r="B6" s="1">
-        <v>45</v>
-      </c>
-      <c r="C6" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
-        <v>57</v>
-      </c>
-      <c r="B7" s="1">
-        <v>25</v>
-      </c>
-      <c r="C7" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
-        <v>58</v>
-      </c>
-      <c r="B8" s="1">
-        <v>420</v>
-      </c>
-      <c r="C8" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A9" t="s">
-        <v>59</v>
-      </c>
-      <c r="B9" s="1">
-        <v>58</v>
-      </c>
-      <c r="C9" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A10" t="s">
-        <v>60</v>
-      </c>
-      <c r="B10" s="1">
-        <v>35</v>
-      </c>
-      <c r="C10" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A11" t="s">
-        <v>61</v>
-      </c>
-      <c r="B11" s="1">
-        <v>28</v>
-      </c>
-      <c r="C11" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A12" t="s">
-        <v>62</v>
-      </c>
-      <c r="B12" s="1">
-        <v>38</v>
-      </c>
-      <c r="C12" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A13" t="s">
-        <v>63</v>
-      </c>
-      <c r="B13" s="1">
-        <v>3112</v>
-      </c>
-      <c r="C13" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A15" t="s">
-        <v>65</v>
-      </c>
-      <c r="B15" s="1">
-        <v>320</v>
-      </c>
-      <c r="C15" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A16" t="s">
-        <v>67</v>
-      </c>
-      <c r="B16" s="1">
-        <v>640</v>
-      </c>
-      <c r="C16" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A17" t="s">
-        <v>69</v>
-      </c>
-      <c r="B17" s="1">
-        <v>168</v>
-      </c>
-      <c r="C17" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A18" t="s">
-        <v>71</v>
-      </c>
-      <c r="B18" s="1">
-        <v>142</v>
-      </c>
-      <c r="C18" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A19" t="s">
-        <v>73</v>
-      </c>
-      <c r="B19" s="1">
-        <v>84</v>
-      </c>
-      <c r="C19" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A20" t="s">
-        <v>74</v>
-      </c>
-      <c r="B20" s="1">
-        <v>220</v>
-      </c>
-      <c r="C20" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A21" t="s">
-        <v>76</v>
-      </c>
-      <c r="B21" s="1">
-        <v>34</v>
-      </c>
-      <c r="C21" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A22" t="s">
-        <v>78</v>
-      </c>
-      <c r="B22" s="1">
-        <v>108</v>
-      </c>
-      <c r="C22" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A23" t="s">
-        <v>80</v>
-      </c>
-      <c r="B23" s="1">
-        <v>1716</v>
-      </c>
-      <c r="C23" t="s">
-        <v>64</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <ignoredErrors>
-    <ignoredError sqref="A1:C23" numberStoredAsText="1"/>
-  </ignoredErrors>
-</worksheet>
 </file>
</xml_diff>